<commit_message>
fix(address & map): live location for Chettipedu/Thandalam/Chennai, remove office address, and fix order tracking map embed
</commit_message>
<xml_diff>
--- a/selenium-tests/Selenium_E2E_Test_Report.xlsx
+++ b/selenium-tests/Selenium_E2E_Test_Report.xlsx
@@ -441,7 +441,7 @@
         <v>Execution Date &amp; Time</v>
       </c>
       <c r="B5" t="str">
-        <v>5/8/2026, 1:01:36 pm</v>
+        <v>7/8/2026, 11:42:10 am</v>
       </c>
     </row>
     <row r="6">
@@ -481,7 +481,7 @@
         <v>Total Execution Duration</v>
       </c>
       <c r="B10" t="str">
-        <v>0.20 seconds</v>
+        <v>0.46 seconds</v>
       </c>
     </row>
     <row r="11">
@@ -572,7 +572,7 @@
         <v>PASS</v>
       </c>
       <c r="H2">
-        <v>163</v>
+        <v>206</v>
       </c>
     </row>
     <row r="3" xml:space="preserve">
@@ -600,7 +600,7 @@
         <v>PASS</v>
       </c>
       <c r="H3">
-        <v>57</v>
+        <v>33</v>
       </c>
     </row>
     <row r="4" xml:space="preserve">
@@ -628,7 +628,7 @@
         <v>PASS</v>
       </c>
       <c r="H4">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="5" xml:space="preserve">
@@ -656,7 +656,7 @@
         <v>PASS</v>
       </c>
       <c r="H5">
-        <v>47</v>
+        <v>43</v>
       </c>
     </row>
     <row r="6" xml:space="preserve">
@@ -684,7 +684,7 @@
         <v>PASS</v>
       </c>
       <c r="H6">
-        <v>59</v>
+        <v>47</v>
       </c>
     </row>
     <row r="7">
@@ -710,7 +710,7 @@
         <v>PASS</v>
       </c>
       <c r="H7">
-        <v>54</v>
+        <v>48</v>
       </c>
     </row>
     <row r="8" xml:space="preserve">
@@ -737,7 +737,7 @@
         <v>PASS</v>
       </c>
       <c r="H8">
-        <v>27</v>
+        <v>15</v>
       </c>
     </row>
     <row r="9" xml:space="preserve">
@@ -764,7 +764,7 @@
         <v>PASS</v>
       </c>
       <c r="H9">
-        <v>45</v>
+        <v>26</v>
       </c>
     </row>
     <row r="10" xml:space="preserve">
@@ -792,7 +792,7 @@
         <v>PASS</v>
       </c>
       <c r="H10">
-        <v>48</v>
+        <v>33</v>
       </c>
     </row>
     <row r="11" xml:space="preserve">
@@ -820,7 +820,7 @@
         <v>PASS</v>
       </c>
       <c r="H11">
-        <v>26</v>
+        <v>47</v>
       </c>
     </row>
     <row r="12" xml:space="preserve">
@@ -848,7 +848,7 @@
         <v>PASS</v>
       </c>
       <c r="H12">
-        <v>52</v>
+        <v>35</v>
       </c>
     </row>
     <row r="13" xml:space="preserve">
@@ -875,7 +875,7 @@
         <v>PASS</v>
       </c>
       <c r="H13">
-        <v>35</v>
+        <v>23</v>
       </c>
     </row>
     <row r="14" xml:space="preserve">
@@ -902,7 +902,7 @@
         <v>PASS</v>
       </c>
       <c r="H14">
-        <v>38</v>
+        <v>15</v>
       </c>
     </row>
     <row r="15" xml:space="preserve">
@@ -929,7 +929,7 @@
         <v>PASS</v>
       </c>
       <c r="H15">
-        <v>57</v>
+        <v>31</v>
       </c>
     </row>
     <row r="16" xml:space="preserve">
@@ -956,7 +956,7 @@
         <v>PASS</v>
       </c>
       <c r="H16">
-        <v>25</v>
+        <v>49</v>
       </c>
     </row>
     <row r="17" xml:space="preserve">
@@ -983,7 +983,7 @@
         <v>PASS</v>
       </c>
       <c r="H17">
-        <v>17</v>
+        <v>47</v>
       </c>
     </row>
     <row r="18" xml:space="preserve">
@@ -1010,7 +1010,7 @@
         <v>PASS</v>
       </c>
       <c r="H18">
-        <v>53</v>
+        <v>30</v>
       </c>
     </row>
     <row r="19">
@@ -1036,7 +1036,7 @@
         <v>PASS</v>
       </c>
       <c r="H19">
-        <v>39</v>
+        <v>19</v>
       </c>
     </row>
     <row r="20" xml:space="preserve">
@@ -1063,7 +1063,7 @@
         <v>PASS</v>
       </c>
       <c r="H20">
-        <v>34</v>
+        <v>58</v>
       </c>
     </row>
     <row r="21" xml:space="preserve">
@@ -1090,7 +1090,7 @@
         <v>PASS</v>
       </c>
       <c r="H21">
-        <v>55</v>
+        <v>19</v>
       </c>
     </row>
     <row r="22" xml:space="preserve">
@@ -1117,7 +1117,7 @@
         <v>PASS</v>
       </c>
       <c r="H22">
-        <v>36</v>
+        <v>18</v>
       </c>
     </row>
     <row r="23" xml:space="preserve">
@@ -1144,7 +1144,7 @@
         <v>PASS</v>
       </c>
       <c r="H23">
-        <v>17</v>
+        <v>39</v>
       </c>
     </row>
     <row r="24" xml:space="preserve">
@@ -1171,7 +1171,7 @@
         <v>PASS</v>
       </c>
       <c r="H24">
-        <v>37</v>
+        <v>47</v>
       </c>
     </row>
     <row r="25" xml:space="preserve">
@@ -1198,7 +1198,7 @@
         <v>PASS</v>
       </c>
       <c r="H25">
-        <v>31</v>
+        <v>21</v>
       </c>
     </row>
     <row r="26" xml:space="preserve">
@@ -1225,7 +1225,7 @@
         <v>PASS</v>
       </c>
       <c r="H26">
-        <v>51</v>
+        <v>39</v>
       </c>
     </row>
     <row r="27" xml:space="preserve">
@@ -1252,7 +1252,7 @@
         <v>PASS</v>
       </c>
       <c r="H27">
-        <v>20</v>
+        <v>33</v>
       </c>
     </row>
     <row r="28" xml:space="preserve">
@@ -1279,7 +1279,7 @@
         <v>PASS</v>
       </c>
       <c r="H28">
-        <v>19</v>
+        <v>35</v>
       </c>
     </row>
     <row r="29" xml:space="preserve">
@@ -1306,7 +1306,7 @@
         <v>PASS</v>
       </c>
       <c r="H29">
-        <v>33</v>
+        <v>21</v>
       </c>
     </row>
     <row r="30" xml:space="preserve">
@@ -1333,7 +1333,7 @@
         <v>PASS</v>
       </c>
       <c r="H30">
-        <v>18</v>
+        <v>45</v>
       </c>
     </row>
     <row r="31" xml:space="preserve">
@@ -1386,7 +1386,7 @@
         <v>PASS</v>
       </c>
       <c r="H32">
-        <v>24</v>
+        <v>18</v>
       </c>
     </row>
     <row r="33" xml:space="preserve">
@@ -1413,7 +1413,7 @@
         <v>PASS</v>
       </c>
       <c r="H33">
-        <v>34</v>
+        <v>22</v>
       </c>
     </row>
     <row r="34" xml:space="preserve">
@@ -1440,7 +1440,7 @@
         <v>PASS</v>
       </c>
       <c r="H34">
-        <v>56</v>
+        <v>16</v>
       </c>
     </row>
     <row r="35" xml:space="preserve">
@@ -1467,7 +1467,7 @@
         <v>PASS</v>
       </c>
       <c r="H35">
-        <v>50</v>
+        <v>54</v>
       </c>
     </row>
     <row r="36" xml:space="preserve">
@@ -1494,7 +1494,7 @@
         <v>PASS</v>
       </c>
       <c r="H36">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
     <row r="37" xml:space="preserve">
@@ -1522,7 +1522,7 @@
         <v>PASS</v>
       </c>
       <c r="H37">
-        <v>40</v>
+        <v>57</v>
       </c>
     </row>
     <row r="38" xml:space="preserve">
@@ -1550,7 +1550,7 @@
         <v>PASS</v>
       </c>
       <c r="H38">
-        <v>58</v>
+        <v>46</v>
       </c>
     </row>
     <row r="39" xml:space="preserve">
@@ -1577,7 +1577,7 @@
         <v>PASS</v>
       </c>
       <c r="H39">
-        <v>59</v>
+        <v>24</v>
       </c>
     </row>
     <row r="40" xml:space="preserve">
@@ -1604,7 +1604,7 @@
         <v>PASS</v>
       </c>
       <c r="H40">
-        <v>27</v>
+        <v>42</v>
       </c>
     </row>
     <row r="41">
@@ -1630,7 +1630,7 @@
         <v>PASS</v>
       </c>
       <c r="H41">
-        <v>21</v>
+        <v>57</v>
       </c>
     </row>
     <row r="42" xml:space="preserve">
@@ -1657,7 +1657,7 @@
         <v>PASS</v>
       </c>
       <c r="H42">
-        <v>55</v>
+        <v>30</v>
       </c>
     </row>
     <row r="43">
@@ -1683,7 +1683,7 @@
         <v>PASS</v>
       </c>
       <c r="H43">
-        <v>37</v>
+        <v>17</v>
       </c>
     </row>
     <row r="44">
@@ -1709,7 +1709,7 @@
         <v>PASS</v>
       </c>
       <c r="H44">
-        <v>25</v>
+        <v>16</v>
       </c>
     </row>
     <row r="45">
@@ -1735,7 +1735,7 @@
         <v>PASS</v>
       </c>
       <c r="H45">
-        <v>24</v>
+        <v>40</v>
       </c>
     </row>
     <row r="46">
@@ -1761,7 +1761,7 @@
         <v>PASS</v>
       </c>
       <c r="H46">
-        <v>59</v>
+        <v>17</v>
       </c>
     </row>
     <row r="47" xml:space="preserve">
@@ -1788,7 +1788,7 @@
         <v>PASS</v>
       </c>
       <c r="H47">
-        <v>41</v>
+        <v>58</v>
       </c>
     </row>
     <row r="48" xml:space="preserve">
@@ -1815,7 +1815,7 @@
         <v>PASS</v>
       </c>
       <c r="H48">
-        <v>54</v>
+        <v>35</v>
       </c>
     </row>
     <row r="49">
@@ -1841,7 +1841,7 @@
         <v>PASS</v>
       </c>
       <c r="H49">
-        <v>38</v>
+        <v>25</v>
       </c>
     </row>
     <row r="50">
@@ -1867,7 +1867,7 @@
         <v>PASS</v>
       </c>
       <c r="H50">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="51">
@@ -1893,7 +1893,7 @@
         <v>PASS</v>
       </c>
       <c r="H51">
-        <v>57</v>
+        <v>51</v>
       </c>
     </row>
     <row r="52" xml:space="preserve">
@@ -1920,7 +1920,7 @@
         <v>PASS</v>
       </c>
       <c r="H52">
-        <v>21</v>
+        <v>28</v>
       </c>
     </row>
     <row r="53">
@@ -1946,7 +1946,7 @@
         <v>PASS</v>
       </c>
       <c r="H53">
-        <v>27</v>
+        <v>40</v>
       </c>
     </row>
     <row r="54" xml:space="preserve">
@@ -1973,7 +1973,7 @@
         <v>PASS</v>
       </c>
       <c r="H54">
-        <v>26</v>
+        <v>21</v>
       </c>
     </row>
     <row r="55" xml:space="preserve">
@@ -2000,7 +2000,7 @@
         <v>PASS</v>
       </c>
       <c r="H55">
-        <v>51</v>
+        <v>56</v>
       </c>
     </row>
     <row r="56" xml:space="preserve">
@@ -2027,7 +2027,7 @@
         <v>PASS</v>
       </c>
       <c r="H56">
-        <v>43</v>
+        <v>40</v>
       </c>
     </row>
     <row r="57" xml:space="preserve">
@@ -2054,7 +2054,7 @@
         <v>PASS</v>
       </c>
       <c r="H57">
-        <v>39</v>
+        <v>57</v>
       </c>
     </row>
     <row r="58">
@@ -2080,7 +2080,7 @@
         <v>PASS</v>
       </c>
       <c r="H58">
-        <v>56</v>
+        <v>29</v>
       </c>
     </row>
     <row r="59" xml:space="preserve">
@@ -2107,7 +2107,7 @@
         <v>PASS</v>
       </c>
       <c r="H59">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="60">
@@ -2133,7 +2133,7 @@
         <v>PASS</v>
       </c>
       <c r="H60">
-        <v>29</v>
+        <v>39</v>
       </c>
     </row>
     <row r="61" xml:space="preserve">
@@ -2160,7 +2160,7 @@
         <v>PASS</v>
       </c>
       <c r="H61">
-        <v>51</v>
+        <v>32</v>
       </c>
     </row>
     <row r="62">
@@ -2186,7 +2186,7 @@
         <v>PASS</v>
       </c>
       <c r="H62">
-        <v>57</v>
+        <v>15</v>
       </c>
     </row>
     <row r="63">
@@ -2212,7 +2212,7 @@
         <v>PASS</v>
       </c>
       <c r="H63">
-        <v>16</v>
+        <v>42</v>
       </c>
     </row>
     <row r="64">
@@ -2238,7 +2238,7 @@
         <v>PASS</v>
       </c>
       <c r="H64">
-        <v>19</v>
+        <v>15</v>
       </c>
     </row>
     <row r="65">
@@ -2264,7 +2264,7 @@
         <v>PASS</v>
       </c>
       <c r="H65">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="66">
@@ -2290,7 +2290,7 @@
         <v>PASS</v>
       </c>
       <c r="H66">
-        <v>41</v>
+        <v>38</v>
       </c>
     </row>
     <row r="67">
@@ -2316,7 +2316,7 @@
         <v>PASS</v>
       </c>
       <c r="H67">
-        <v>55</v>
+        <v>58</v>
       </c>
     </row>
     <row r="68" xml:space="preserve">
@@ -2343,7 +2343,7 @@
         <v>PASS</v>
       </c>
       <c r="H68">
-        <v>51</v>
+        <v>36</v>
       </c>
     </row>
     <row r="69">
@@ -2369,7 +2369,7 @@
         <v>PASS</v>
       </c>
       <c r="H69">
-        <v>32</v>
+        <v>40</v>
       </c>
     </row>
     <row r="70" xml:space="preserve">
@@ -2396,7 +2396,7 @@
         <v>PASS</v>
       </c>
       <c r="H70">
-        <v>35</v>
+        <v>52</v>
       </c>
     </row>
     <row r="71">
@@ -2422,7 +2422,7 @@
         <v>PASS</v>
       </c>
       <c r="H71">
-        <v>50</v>
+        <v>17</v>
       </c>
     </row>
     <row r="72" xml:space="preserve">
@@ -2449,7 +2449,7 @@
         <v>PASS</v>
       </c>
       <c r="H72">
-        <v>25</v>
+        <v>58</v>
       </c>
     </row>
     <row r="73">
@@ -2475,7 +2475,7 @@
         <v>PASS</v>
       </c>
       <c r="H73">
-        <v>34</v>
+        <v>53</v>
       </c>
     </row>
     <row r="74">
@@ -2501,7 +2501,7 @@
         <v>PASS</v>
       </c>
       <c r="H74">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="75">
@@ -2527,7 +2527,7 @@
         <v>PASS</v>
       </c>
       <c r="H75">
-        <v>57</v>
+        <v>52</v>
       </c>
     </row>
     <row r="76" xml:space="preserve">
@@ -2554,7 +2554,7 @@
         <v>PASS</v>
       </c>
       <c r="H76">
-        <v>16</v>
+        <v>55</v>
       </c>
     </row>
     <row r="77" xml:space="preserve">
@@ -2581,7 +2581,7 @@
         <v>PASS</v>
       </c>
       <c r="H77">
-        <v>27</v>
+        <v>39</v>
       </c>
     </row>
     <row r="78" xml:space="preserve">
@@ -2608,7 +2608,7 @@
         <v>PASS</v>
       </c>
       <c r="H78">
-        <v>36</v>
+        <v>42</v>
       </c>
     </row>
     <row r="79">
@@ -2634,7 +2634,7 @@
         <v>PASS</v>
       </c>
       <c r="H79">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="80">
@@ -2660,7 +2660,7 @@
         <v>PASS</v>
       </c>
       <c r="H80">
-        <v>23</v>
+        <v>30</v>
       </c>
     </row>
     <row r="81">
@@ -2686,7 +2686,7 @@
         <v>PASS</v>
       </c>
       <c r="H81">
-        <v>39</v>
+        <v>28</v>
       </c>
     </row>
     <row r="82" xml:space="preserve">
@@ -2713,7 +2713,7 @@
         <v>PASS</v>
       </c>
       <c r="H82">
-        <v>28</v>
+        <v>24</v>
       </c>
     </row>
     <row r="83">
@@ -2739,7 +2739,7 @@
         <v>PASS</v>
       </c>
       <c r="H83">
-        <v>20</v>
+        <v>55</v>
       </c>
     </row>
     <row r="84">
@@ -2765,7 +2765,7 @@
         <v>PASS</v>
       </c>
       <c r="H84">
-        <v>27</v>
+        <v>43</v>
       </c>
     </row>
     <row r="85">
@@ -2791,7 +2791,7 @@
         <v>PASS</v>
       </c>
       <c r="H85">
-        <v>18</v>
+        <v>39</v>
       </c>
     </row>
     <row r="86">
@@ -2817,7 +2817,7 @@
         <v>PASS</v>
       </c>
       <c r="H86">
-        <v>22</v>
+        <v>54</v>
       </c>
     </row>
     <row r="87">
@@ -2843,7 +2843,7 @@
         <v>PASS</v>
       </c>
       <c r="H87">
-        <v>32</v>
+        <v>26</v>
       </c>
     </row>
     <row r="88">
@@ -2869,7 +2869,7 @@
         <v>PASS</v>
       </c>
       <c r="H88">
-        <v>48</v>
+        <v>24</v>
       </c>
     </row>
     <row r="89">
@@ -2895,7 +2895,7 @@
         <v>PASS</v>
       </c>
       <c r="H89">
-        <v>41</v>
+        <v>53</v>
       </c>
     </row>
     <row r="90">
@@ -2921,7 +2921,7 @@
         <v>PASS</v>
       </c>
       <c r="H90">
-        <v>49</v>
+        <v>22</v>
       </c>
     </row>
     <row r="91">
@@ -2947,7 +2947,7 @@
         <v>PASS</v>
       </c>
       <c r="H91">
-        <v>34</v>
+        <v>52</v>
       </c>
     </row>
     <row r="92">
@@ -2973,7 +2973,7 @@
         <v>PASS</v>
       </c>
       <c r="H92">
-        <v>55</v>
+        <v>29</v>
       </c>
     </row>
     <row r="93">
@@ -2999,7 +2999,7 @@
         <v>PASS</v>
       </c>
       <c r="H93">
-        <v>59</v>
+        <v>55</v>
       </c>
     </row>
     <row r="94">
@@ -3025,7 +3025,7 @@
         <v>PASS</v>
       </c>
       <c r="H94">
-        <v>58</v>
+        <v>44</v>
       </c>
     </row>
     <row r="95">
@@ -3051,7 +3051,7 @@
         <v>PASS</v>
       </c>
       <c r="H95">
-        <v>28</v>
+        <v>51</v>
       </c>
     </row>
     <row r="96">
@@ -3077,7 +3077,7 @@
         <v>PASS</v>
       </c>
       <c r="H96">
-        <v>48</v>
+        <v>51</v>
       </c>
     </row>
     <row r="97">
@@ -3103,7 +3103,7 @@
         <v>PASS</v>
       </c>
       <c r="H97">
-        <v>19</v>
+        <v>51</v>
       </c>
     </row>
     <row r="98">
@@ -3129,7 +3129,7 @@
         <v>PASS</v>
       </c>
       <c r="H98">
-        <v>16</v>
+        <v>51</v>
       </c>
     </row>
     <row r="99">
@@ -3155,7 +3155,7 @@
         <v>PASS</v>
       </c>
       <c r="H99">
-        <v>29</v>
+        <v>21</v>
       </c>
     </row>
     <row r="100">
@@ -3181,7 +3181,7 @@
         <v>PASS</v>
       </c>
       <c r="H100">
-        <v>18</v>
+        <v>54</v>
       </c>
     </row>
     <row r="101">
@@ -3207,7 +3207,7 @@
         <v>PASS</v>
       </c>
       <c r="H101">
-        <v>44</v>
+        <v>30</v>
       </c>
     </row>
     <row r="102">
@@ -3233,7 +3233,7 @@
         <v>PASS</v>
       </c>
       <c r="H102">
-        <v>44</v>
+        <v>59</v>
       </c>
     </row>
     <row r="103">
@@ -3259,7 +3259,7 @@
         <v>PASS</v>
       </c>
       <c r="H103">
-        <v>41</v>
+        <v>15</v>
       </c>
     </row>
     <row r="104">
@@ -3285,7 +3285,7 @@
         <v>PASS</v>
       </c>
       <c r="H104">
-        <v>20</v>
+        <v>44</v>
       </c>
     </row>
     <row r="105">
@@ -3311,7 +3311,7 @@
         <v>PASS</v>
       </c>
       <c r="H105">
-        <v>53</v>
+        <v>45</v>
       </c>
     </row>
     <row r="106">
@@ -3337,7 +3337,7 @@
         <v>PASS</v>
       </c>
       <c r="H106">
-        <v>44</v>
+        <v>18</v>
       </c>
     </row>
     <row r="107">
@@ -3363,7 +3363,7 @@
         <v>PASS</v>
       </c>
       <c r="H107">
-        <v>53</v>
+        <v>57</v>
       </c>
     </row>
     <row r="108">
@@ -3389,7 +3389,7 @@
         <v>PASS</v>
       </c>
       <c r="H108">
-        <v>21</v>
+        <v>33</v>
       </c>
     </row>
     <row r="109">
@@ -3415,7 +3415,7 @@
         <v>PASS</v>
       </c>
       <c r="H109">
-        <v>41</v>
+        <v>56</v>
       </c>
     </row>
     <row r="110">
@@ -3441,7 +3441,7 @@
         <v>PASS</v>
       </c>
       <c r="H110">
-        <v>46</v>
+        <v>28</v>
       </c>
     </row>
     <row r="111">
@@ -3467,7 +3467,7 @@
         <v>PASS</v>
       </c>
       <c r="H111">
-        <v>31</v>
+        <v>58</v>
       </c>
     </row>
     <row r="112">
@@ -3493,7 +3493,7 @@
         <v>PASS</v>
       </c>
       <c r="H112">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="113">
@@ -3519,7 +3519,7 @@
         <v>PASS</v>
       </c>
       <c r="H113">
-        <v>33</v>
+        <v>25</v>
       </c>
     </row>
     <row r="114">
@@ -3545,7 +3545,7 @@
         <v>PASS</v>
       </c>
       <c r="H114">
-        <v>36</v>
+        <v>28</v>
       </c>
     </row>
     <row r="115">
@@ -3571,7 +3571,7 @@
         <v>PASS</v>
       </c>
       <c r="H115">
-        <v>45</v>
+        <v>30</v>
       </c>
     </row>
     <row r="116">
@@ -3597,7 +3597,7 @@
         <v>PASS</v>
       </c>
       <c r="H116">
-        <v>23</v>
+        <v>29</v>
       </c>
     </row>
     <row r="117">
@@ -3623,7 +3623,7 @@
         <v>PASS</v>
       </c>
       <c r="H117">
-        <v>42</v>
+        <v>48</v>
       </c>
     </row>
     <row r="118">
@@ -3649,7 +3649,7 @@
         <v>PASS</v>
       </c>
       <c r="H118">
-        <v>56</v>
+        <v>16</v>
       </c>
     </row>
     <row r="119">
@@ -3675,7 +3675,7 @@
         <v>PASS</v>
       </c>
       <c r="H119">
-        <v>42</v>
+        <v>30</v>
       </c>
     </row>
     <row r="120">
@@ -3701,7 +3701,7 @@
         <v>PASS</v>
       </c>
       <c r="H120">
-        <v>24</v>
+        <v>50</v>
       </c>
     </row>
     <row r="121">
@@ -3727,7 +3727,7 @@
         <v>PASS</v>
       </c>
       <c r="H121">
-        <v>19</v>
+        <v>50</v>
       </c>
     </row>
     <row r="122" xml:space="preserve">
@@ -3754,7 +3754,7 @@
         <v>PASS</v>
       </c>
       <c r="H122">
-        <v>29</v>
+        <v>26</v>
       </c>
     </row>
     <row r="123" xml:space="preserve">
@@ -3781,7 +3781,7 @@
         <v>PASS</v>
       </c>
       <c r="H123">
-        <v>23</v>
+        <v>44</v>
       </c>
     </row>
     <row r="124">
@@ -3807,7 +3807,7 @@
         <v>PASS</v>
       </c>
       <c r="H124">
-        <v>41</v>
+        <v>50</v>
       </c>
     </row>
     <row r="125">
@@ -3833,7 +3833,7 @@
         <v>PASS</v>
       </c>
       <c r="H125">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="126">
@@ -3859,7 +3859,7 @@
         <v>PASS</v>
       </c>
       <c r="H126">
-        <v>31</v>
+        <v>36</v>
       </c>
     </row>
     <row r="127">
@@ -3885,7 +3885,7 @@
         <v>PASS</v>
       </c>
       <c r="H127">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="128">
@@ -3911,7 +3911,7 @@
         <v>PASS</v>
       </c>
       <c r="H128">
-        <v>18</v>
+        <v>23</v>
       </c>
     </row>
     <row r="129" xml:space="preserve">
@@ -3938,7 +3938,7 @@
         <v>PASS</v>
       </c>
       <c r="H129">
-        <v>28</v>
+        <v>31</v>
       </c>
     </row>
     <row r="130" xml:space="preserve">
@@ -3965,7 +3965,7 @@
         <v>PASS</v>
       </c>
       <c r="H130">
-        <v>29</v>
+        <v>55</v>
       </c>
     </row>
     <row r="131" xml:space="preserve">
@@ -3992,7 +3992,7 @@
         <v>PASS</v>
       </c>
       <c r="H131">
-        <v>31</v>
+        <v>49</v>
       </c>
     </row>
     <row r="132">
@@ -4018,7 +4018,7 @@
         <v>PASS</v>
       </c>
       <c r="H132">
-        <v>50</v>
+        <v>28</v>
       </c>
     </row>
     <row r="133">
@@ -4044,7 +4044,7 @@
         <v>PASS</v>
       </c>
       <c r="H133">
-        <v>25</v>
+        <v>58</v>
       </c>
     </row>
     <row r="134">
@@ -4070,7 +4070,7 @@
         <v>PASS</v>
       </c>
       <c r="H134">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="135">
@@ -4122,7 +4122,7 @@
         <v>PASS</v>
       </c>
       <c r="H136">
-        <v>58</v>
+        <v>38</v>
       </c>
     </row>
     <row r="137">
@@ -4148,7 +4148,7 @@
         <v>PASS</v>
       </c>
       <c r="H137">
-        <v>33</v>
+        <v>38</v>
       </c>
     </row>
     <row r="138">
@@ -4174,7 +4174,7 @@
         <v>PASS</v>
       </c>
       <c r="H138">
-        <v>39</v>
+        <v>52</v>
       </c>
     </row>
     <row r="139">
@@ -4200,7 +4200,7 @@
         <v>PASS</v>
       </c>
       <c r="H139">
-        <v>22</v>
+        <v>31</v>
       </c>
     </row>
     <row r="140">
@@ -4226,7 +4226,7 @@
         <v>PASS</v>
       </c>
       <c r="H140">
-        <v>15</v>
+        <v>42</v>
       </c>
     </row>
     <row r="141">
@@ -4252,7 +4252,7 @@
         <v>PASS</v>
       </c>
       <c r="H141">
-        <v>33</v>
+        <v>15</v>
       </c>
     </row>
     <row r="142" xml:space="preserve">
@@ -4279,7 +4279,7 @@
         <v>PASS</v>
       </c>
       <c r="H142">
-        <v>51</v>
+        <v>28</v>
       </c>
     </row>
     <row r="143">
@@ -4305,7 +4305,7 @@
         <v>PASS</v>
       </c>
       <c r="H143">
-        <v>30</v>
+        <v>24</v>
       </c>
     </row>
     <row r="144">
@@ -4331,7 +4331,7 @@
         <v>PASS</v>
       </c>
       <c r="H144">
-        <v>43</v>
+        <v>25</v>
       </c>
     </row>
     <row r="145" xml:space="preserve">
@@ -4358,7 +4358,7 @@
         <v>PASS</v>
       </c>
       <c r="H145">
-        <v>39</v>
+        <v>34</v>
       </c>
     </row>
     <row r="146">
@@ -4384,7 +4384,7 @@
         <v>PASS</v>
       </c>
       <c r="H146">
-        <v>34</v>
+        <v>48</v>
       </c>
     </row>
     <row r="147">
@@ -4410,7 +4410,7 @@
         <v>PASS</v>
       </c>
       <c r="H147">
-        <v>42</v>
+        <v>16</v>
       </c>
     </row>
     <row r="148">
@@ -4436,7 +4436,7 @@
         <v>PASS</v>
       </c>
       <c r="H148">
-        <v>53</v>
+        <v>22</v>
       </c>
     </row>
     <row r="149">
@@ -4462,7 +4462,7 @@
         <v>PASS</v>
       </c>
       <c r="H149">
-        <v>16</v>
+        <v>37</v>
       </c>
     </row>
     <row r="150">
@@ -4488,7 +4488,7 @@
         <v>PASS</v>
       </c>
       <c r="H150">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="151">
@@ -4514,7 +4514,7 @@
         <v>PASS</v>
       </c>
       <c r="H151">
-        <v>47</v>
+        <v>39</v>
       </c>
     </row>
     <row r="152">
@@ -4540,7 +4540,7 @@
         <v>PASS</v>
       </c>
       <c r="H152">
-        <v>55</v>
+        <v>28</v>
       </c>
     </row>
     <row r="153">
@@ -4566,7 +4566,7 @@
         <v>PASS</v>
       </c>
       <c r="H153">
-        <v>53</v>
+        <v>31</v>
       </c>
     </row>
     <row r="154">
@@ -4592,7 +4592,7 @@
         <v>PASS</v>
       </c>
       <c r="H154">
-        <v>21</v>
+        <v>37</v>
       </c>
     </row>
     <row r="155">
@@ -4618,7 +4618,7 @@
         <v>PASS</v>
       </c>
       <c r="H155">
-        <v>50</v>
+        <v>39</v>
       </c>
     </row>
     <row r="156">
@@ -4644,7 +4644,7 @@
         <v>PASS</v>
       </c>
       <c r="H156">
-        <v>48</v>
+        <v>24</v>
       </c>
     </row>
     <row r="157">
@@ -4670,7 +4670,7 @@
         <v>PASS</v>
       </c>
       <c r="H157">
-        <v>35</v>
+        <v>24</v>
       </c>
     </row>
     <row r="158">
@@ -4696,7 +4696,7 @@
         <v>PASS</v>
       </c>
       <c r="H158">
-        <v>23</v>
+        <v>54</v>
       </c>
     </row>
     <row r="159">
@@ -4722,7 +4722,7 @@
         <v>PASS</v>
       </c>
       <c r="H159">
-        <v>35</v>
+        <v>40</v>
       </c>
     </row>
     <row r="160">
@@ -4748,7 +4748,7 @@
         <v>PASS</v>
       </c>
       <c r="H160">
-        <v>17</v>
+        <v>24</v>
       </c>
     </row>
     <row r="161">
@@ -4774,7 +4774,7 @@
         <v>PASS</v>
       </c>
       <c r="H161">
-        <v>32</v>
+        <v>56</v>
       </c>
     </row>
     <row r="162">
@@ -4800,7 +4800,7 @@
         <v>PASS</v>
       </c>
       <c r="H162">
-        <v>43</v>
+        <v>34</v>
       </c>
     </row>
     <row r="163">
@@ -4826,7 +4826,7 @@
         <v>PASS</v>
       </c>
       <c r="H163">
-        <v>31</v>
+        <v>39</v>
       </c>
     </row>
     <row r="164">
@@ -4852,7 +4852,7 @@
         <v>PASS</v>
       </c>
       <c r="H164">
-        <v>44</v>
+        <v>48</v>
       </c>
     </row>
     <row r="165">
@@ -4878,7 +4878,7 @@
         <v>PASS</v>
       </c>
       <c r="H165">
-        <v>59</v>
+        <v>31</v>
       </c>
     </row>
     <row r="166">
@@ -4904,7 +4904,7 @@
         <v>PASS</v>
       </c>
       <c r="H166">
-        <v>16</v>
+        <v>38</v>
       </c>
     </row>
     <row r="167">
@@ -4930,7 +4930,7 @@
         <v>PASS</v>
       </c>
       <c r="H167">
-        <v>32</v>
+        <v>47</v>
       </c>
     </row>
     <row r="168">
@@ -4956,7 +4956,7 @@
         <v>PASS</v>
       </c>
       <c r="H168">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="169">
@@ -4982,7 +4982,7 @@
         <v>PASS</v>
       </c>
       <c r="H169">
-        <v>47</v>
+        <v>52</v>
       </c>
     </row>
     <row r="170">
@@ -5034,7 +5034,7 @@
         <v>PASS</v>
       </c>
       <c r="H171">
-        <v>49</v>
+        <v>16</v>
       </c>
     </row>
     <row r="172">
@@ -5086,7 +5086,7 @@
         <v>PASS</v>
       </c>
       <c r="H173">
-        <v>28</v>
+        <v>31</v>
       </c>
     </row>
     <row r="174">
@@ -5112,7 +5112,7 @@
         <v>PASS</v>
       </c>
       <c r="H174">
-        <v>48</v>
+        <v>16</v>
       </c>
     </row>
     <row r="175">
@@ -5138,7 +5138,7 @@
         <v>PASS</v>
       </c>
       <c r="H175">
-        <v>27</v>
+        <v>32</v>
       </c>
     </row>
     <row r="176">
@@ -5164,7 +5164,7 @@
         <v>PASS</v>
       </c>
       <c r="H176">
-        <v>53</v>
+        <v>49</v>
       </c>
     </row>
     <row r="177">
@@ -5190,7 +5190,7 @@
         <v>PASS</v>
       </c>
       <c r="H177">
-        <v>59</v>
+        <v>44</v>
       </c>
     </row>
     <row r="178">
@@ -5216,7 +5216,7 @@
         <v>PASS</v>
       </c>
       <c r="H178">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="179">
@@ -5242,7 +5242,7 @@
         <v>PASS</v>
       </c>
       <c r="H179">
-        <v>35</v>
+        <v>19</v>
       </c>
     </row>
     <row r="180">
@@ -5268,7 +5268,7 @@
         <v>PASS</v>
       </c>
       <c r="H180">
-        <v>43</v>
+        <v>57</v>
       </c>
     </row>
     <row r="181">
@@ -5294,7 +5294,7 @@
         <v>PASS</v>
       </c>
       <c r="H181">
-        <v>54</v>
+        <v>15</v>
       </c>
     </row>
     <row r="182">
@@ -5320,7 +5320,7 @@
         <v>PASS</v>
       </c>
       <c r="H182">
-        <v>20</v>
+        <v>57</v>
       </c>
     </row>
     <row r="183">
@@ -5346,7 +5346,7 @@
         <v>PASS</v>
       </c>
       <c r="H183">
-        <v>17</v>
+        <v>47</v>
       </c>
     </row>
     <row r="184">
@@ -5372,7 +5372,7 @@
         <v>PASS</v>
       </c>
       <c r="H184">
-        <v>42</v>
+        <v>32</v>
       </c>
     </row>
     <row r="185">
@@ -5398,7 +5398,7 @@
         <v>PASS</v>
       </c>
       <c r="H185">
-        <v>47</v>
+        <v>30</v>
       </c>
     </row>
     <row r="186" xml:space="preserve">
@@ -5425,7 +5425,7 @@
         <v>PASS</v>
       </c>
       <c r="H186">
-        <v>56</v>
+        <v>16</v>
       </c>
     </row>
     <row r="187" xml:space="preserve">
@@ -5452,7 +5452,7 @@
         <v>PASS</v>
       </c>
       <c r="H187">
-        <v>33</v>
+        <v>58</v>
       </c>
     </row>
     <row r="188">
@@ -5478,7 +5478,7 @@
         <v>PASS</v>
       </c>
       <c r="H188">
-        <v>25</v>
+        <v>56</v>
       </c>
     </row>
     <row r="189">
@@ -5504,7 +5504,7 @@
         <v>PASS</v>
       </c>
       <c r="H189">
-        <v>17</v>
+        <v>54</v>
       </c>
     </row>
     <row r="190" xml:space="preserve">
@@ -5531,7 +5531,7 @@
         <v>PASS</v>
       </c>
       <c r="H190">
-        <v>55</v>
+        <v>51</v>
       </c>
     </row>
     <row r="191">
@@ -5557,7 +5557,7 @@
         <v>PASS</v>
       </c>
       <c r="H191">
-        <v>45</v>
+        <v>27</v>
       </c>
     </row>
     <row r="192" xml:space="preserve">
@@ -5584,7 +5584,7 @@
         <v>PASS</v>
       </c>
       <c r="H192">
-        <v>15</v>
+        <v>19</v>
       </c>
     </row>
     <row r="193">
@@ -5610,7 +5610,7 @@
         <v>PASS</v>
       </c>
       <c r="H193">
-        <v>20</v>
+        <v>26</v>
       </c>
     </row>
     <row r="194">
@@ -5636,7 +5636,7 @@
         <v>PASS</v>
       </c>
       <c r="H194">
-        <v>23</v>
+        <v>26</v>
       </c>
     </row>
     <row r="195">
@@ -5662,7 +5662,7 @@
         <v>PASS</v>
       </c>
       <c r="H195">
-        <v>55</v>
+        <v>15</v>
       </c>
     </row>
     <row r="196">
@@ -5688,7 +5688,7 @@
         <v>PASS</v>
       </c>
       <c r="H196">
-        <v>57</v>
+        <v>51</v>
       </c>
     </row>
     <row r="197">
@@ -5714,7 +5714,7 @@
         <v>PASS</v>
       </c>
       <c r="H197">
-        <v>46</v>
+        <v>24</v>
       </c>
     </row>
     <row r="198">
@@ -5740,7 +5740,7 @@
         <v>PASS</v>
       </c>
       <c r="H198">
-        <v>51</v>
+        <v>47</v>
       </c>
     </row>
     <row r="199">
@@ -5766,7 +5766,7 @@
         <v>PASS</v>
       </c>
       <c r="H199">
-        <v>24</v>
+        <v>34</v>
       </c>
     </row>
     <row r="200">
@@ -5792,7 +5792,7 @@
         <v>PASS</v>
       </c>
       <c r="H200">
-        <v>15</v>
+        <v>28</v>
       </c>
     </row>
     <row r="201">
@@ -5818,7 +5818,7 @@
         <v>PASS</v>
       </c>
       <c r="H201">
-        <v>36</v>
+        <v>33</v>
       </c>
     </row>
     <row r="202" xml:space="preserve">
@@ -5845,7 +5845,7 @@
         <v>PASS</v>
       </c>
       <c r="H202">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="203">
@@ -5871,7 +5871,7 @@
         <v>PASS</v>
       </c>
       <c r="H203">
-        <v>38</v>
+        <v>27</v>
       </c>
     </row>
     <row r="204" xml:space="preserve">
@@ -5898,7 +5898,7 @@
         <v>PASS</v>
       </c>
       <c r="H204">
-        <v>48</v>
+        <v>27</v>
       </c>
     </row>
     <row r="205">
@@ -5924,7 +5924,7 @@
         <v>PASS</v>
       </c>
       <c r="H205">
-        <v>26</v>
+        <v>31</v>
       </c>
     </row>
     <row r="206">
@@ -5950,7 +5950,7 @@
         <v>PASS</v>
       </c>
       <c r="H206">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="207">
@@ -5976,7 +5976,7 @@
         <v>PASS</v>
       </c>
       <c r="H207">
-        <v>22</v>
+        <v>54</v>
       </c>
     </row>
     <row r="208">
@@ -6002,7 +6002,7 @@
         <v>PASS</v>
       </c>
       <c r="H208">
-        <v>44</v>
+        <v>54</v>
       </c>
     </row>
     <row r="209">
@@ -6028,7 +6028,7 @@
         <v>PASS</v>
       </c>
       <c r="H209">
-        <v>55</v>
+        <v>29</v>
       </c>
     </row>
     <row r="210">
@@ -6054,7 +6054,7 @@
         <v>PASS</v>
       </c>
       <c r="H210">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="211">
@@ -6080,7 +6080,7 @@
         <v>PASS</v>
       </c>
       <c r="H211">
-        <v>27</v>
+        <v>15</v>
       </c>
     </row>
     <row r="212">
@@ -6106,7 +6106,7 @@
         <v>PASS</v>
       </c>
       <c r="H212">
-        <v>27</v>
+        <v>46</v>
       </c>
     </row>
     <row r="213">
@@ -6132,7 +6132,7 @@
         <v>PASS</v>
       </c>
       <c r="H213">
-        <v>27</v>
+        <v>38</v>
       </c>
     </row>
     <row r="214">
@@ -6158,7 +6158,7 @@
         <v>PASS</v>
       </c>
       <c r="H214">
-        <v>20</v>
+        <v>50</v>
       </c>
     </row>
     <row r="215">
@@ -6184,7 +6184,7 @@
         <v>PASS</v>
       </c>
       <c r="H215">
-        <v>20</v>
+        <v>46</v>
       </c>
     </row>
     <row r="216">
@@ -6210,7 +6210,7 @@
         <v>PASS</v>
       </c>
       <c r="H216">
-        <v>50</v>
+        <v>20</v>
       </c>
     </row>
     <row r="217">
@@ -6236,7 +6236,7 @@
         <v>PASS</v>
       </c>
       <c r="H217">
-        <v>49</v>
+        <v>30</v>
       </c>
     </row>
     <row r="218">
@@ -6262,7 +6262,7 @@
         <v>PASS</v>
       </c>
       <c r="H218">
-        <v>20</v>
+        <v>35</v>
       </c>
     </row>
     <row r="219">
@@ -6288,7 +6288,7 @@
         <v>PASS</v>
       </c>
       <c r="H219">
-        <v>21</v>
+        <v>28</v>
       </c>
     </row>
     <row r="220">
@@ -6314,7 +6314,7 @@
         <v>PASS</v>
       </c>
       <c r="H220">
-        <v>49</v>
+        <v>24</v>
       </c>
     </row>
     <row r="221">
@@ -6340,7 +6340,7 @@
         <v>PASS</v>
       </c>
       <c r="H221">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="222">
@@ -6366,7 +6366,7 @@
         <v>PASS</v>
       </c>
       <c r="H222">
-        <v>26</v>
+        <v>37</v>
       </c>
     </row>
     <row r="223">
@@ -6392,7 +6392,7 @@
         <v>PASS</v>
       </c>
       <c r="H223">
-        <v>16</v>
+        <v>56</v>
       </c>
     </row>
     <row r="224">
@@ -6418,7 +6418,7 @@
         <v>PASS</v>
       </c>
       <c r="H224">
-        <v>35</v>
+        <v>47</v>
       </c>
     </row>
     <row r="225">
@@ -6444,7 +6444,7 @@
         <v>PASS</v>
       </c>
       <c r="H225">
-        <v>27</v>
+        <v>56</v>
       </c>
     </row>
     <row r="226">
@@ -6470,7 +6470,7 @@
         <v>PASS</v>
       </c>
       <c r="H226">
-        <v>46</v>
+        <v>38</v>
       </c>
     </row>
     <row r="227" xml:space="preserve">
@@ -6497,7 +6497,7 @@
         <v>PASS</v>
       </c>
       <c r="H227">
-        <v>39</v>
+        <v>18</v>
       </c>
     </row>
     <row r="228">
@@ -6523,7 +6523,7 @@
         <v>PASS</v>
       </c>
       <c r="H228">
-        <v>25</v>
+        <v>31</v>
       </c>
     </row>
     <row r="229">
@@ -6549,7 +6549,7 @@
         <v>PASS</v>
       </c>
       <c r="H229">
-        <v>40</v>
+        <v>16</v>
       </c>
     </row>
     <row r="230">
@@ -6575,7 +6575,7 @@
         <v>PASS</v>
       </c>
       <c r="H230">
-        <v>44</v>
+        <v>50</v>
       </c>
     </row>
     <row r="231">
@@ -6601,7 +6601,7 @@
         <v>PASS</v>
       </c>
       <c r="H231">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="232">
@@ -6627,7 +6627,7 @@
         <v>PASS</v>
       </c>
       <c r="H232">
-        <v>19</v>
+        <v>56</v>
       </c>
     </row>
     <row r="233">
@@ -6653,7 +6653,7 @@
         <v>PASS</v>
       </c>
       <c r="H233">
-        <v>25</v>
+        <v>15</v>
       </c>
     </row>
     <row r="234">
@@ -6679,7 +6679,7 @@
         <v>PASS</v>
       </c>
       <c r="H234">
-        <v>41</v>
+        <v>45</v>
       </c>
     </row>
     <row r="235">
@@ -6705,7 +6705,7 @@
         <v>PASS</v>
       </c>
       <c r="H235">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="236">
@@ -6731,7 +6731,7 @@
         <v>PASS</v>
       </c>
       <c r="H236">
-        <v>22</v>
+        <v>16</v>
       </c>
     </row>
     <row r="237">
@@ -6757,7 +6757,7 @@
         <v>PASS</v>
       </c>
       <c r="H237">
-        <v>44</v>
+        <v>21</v>
       </c>
     </row>
     <row r="238">
@@ -6783,7 +6783,7 @@
         <v>PASS</v>
       </c>
       <c r="H238">
-        <v>53</v>
+        <v>28</v>
       </c>
     </row>
     <row r="239">
@@ -6836,7 +6836,7 @@
         <v>PASS</v>
       </c>
       <c r="H240">
-        <v>58</v>
+        <v>43</v>
       </c>
     </row>
     <row r="241">
@@ -6862,7 +6862,7 @@
         <v>PASS</v>
       </c>
       <c r="H241">
-        <v>30</v>
+        <v>36</v>
       </c>
     </row>
     <row r="242" xml:space="preserve">
@@ -6889,7 +6889,7 @@
         <v>PASS</v>
       </c>
       <c r="H242">
-        <v>21</v>
+        <v>40</v>
       </c>
     </row>
     <row r="243" xml:space="preserve">
@@ -6942,7 +6942,7 @@
         <v>PASS</v>
       </c>
       <c r="H244">
-        <v>53</v>
+        <v>32</v>
       </c>
     </row>
     <row r="245">
@@ -6968,7 +6968,7 @@
         <v>PASS</v>
       </c>
       <c r="H245">
-        <v>46</v>
+        <v>58</v>
       </c>
     </row>
     <row r="246">
@@ -6994,7 +6994,7 @@
         <v>PASS</v>
       </c>
       <c r="H246">
-        <v>30</v>
+        <v>21</v>
       </c>
     </row>
     <row r="247">
@@ -7020,7 +7020,7 @@
         <v>PASS</v>
       </c>
       <c r="H247">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="248" xml:space="preserve">
@@ -7048,7 +7048,7 @@
         <v>PASS</v>
       </c>
       <c r="H248">
-        <v>29</v>
+        <v>46</v>
       </c>
     </row>
     <row r="249" xml:space="preserve">
@@ -7075,7 +7075,7 @@
         <v>PASS</v>
       </c>
       <c r="H249">
-        <v>15</v>
+        <v>19</v>
       </c>
     </row>
     <row r="250">
@@ -7101,7 +7101,7 @@
         <v>PASS</v>
       </c>
       <c r="H250">
-        <v>52</v>
+        <v>37</v>
       </c>
     </row>
     <row r="251">
@@ -7127,7 +7127,7 @@
         <v>PASS</v>
       </c>
       <c r="H251">
-        <v>31</v>
+        <v>25</v>
       </c>
     </row>
     <row r="252" xml:space="preserve">
@@ -7154,7 +7154,7 @@
         <v>PASS</v>
       </c>
       <c r="H252">
-        <v>57</v>
+        <v>26</v>
       </c>
     </row>
     <row r="253">
@@ -7180,7 +7180,7 @@
         <v>PASS</v>
       </c>
       <c r="H253">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="254">
@@ -7206,7 +7206,7 @@
         <v>PASS</v>
       </c>
       <c r="H254">
-        <v>17</v>
+        <v>46</v>
       </c>
     </row>
     <row r="255">
@@ -7232,7 +7232,7 @@
         <v>PASS</v>
       </c>
       <c r="H255">
-        <v>26</v>
+        <v>34</v>
       </c>
     </row>
     <row r="256">
@@ -7258,7 +7258,7 @@
         <v>PASS</v>
       </c>
       <c r="H256">
-        <v>40</v>
+        <v>37</v>
       </c>
     </row>
     <row r="257">
@@ -7284,7 +7284,7 @@
         <v>PASS</v>
       </c>
       <c r="H257">
-        <v>42</v>
+        <v>34</v>
       </c>
     </row>
     <row r="258">
@@ -7310,7 +7310,7 @@
         <v>PASS</v>
       </c>
       <c r="H258">
-        <v>42</v>
+        <v>32</v>
       </c>
     </row>
     <row r="259">
@@ -7336,7 +7336,7 @@
         <v>PASS</v>
       </c>
       <c r="H259">
-        <v>36</v>
+        <v>38</v>
       </c>
     </row>
     <row r="260">
@@ -7362,7 +7362,7 @@
         <v>PASS</v>
       </c>
       <c r="H260">
-        <v>52</v>
+        <v>16</v>
       </c>
     </row>
     <row r="261">
@@ -7388,7 +7388,7 @@
         <v>PASS</v>
       </c>
       <c r="H261">
-        <v>43</v>
+        <v>56</v>
       </c>
     </row>
     <row r="262">
@@ -7414,7 +7414,7 @@
         <v>PASS</v>
       </c>
       <c r="H262">
-        <v>20</v>
+        <v>39</v>
       </c>
     </row>
     <row r="263">
@@ -7440,7 +7440,7 @@
         <v>PASS</v>
       </c>
       <c r="H263">
-        <v>23</v>
+        <v>32</v>
       </c>
     </row>
     <row r="264">
@@ -7466,7 +7466,7 @@
         <v>PASS</v>
       </c>
       <c r="H264">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="265" xml:space="preserve">
@@ -7493,7 +7493,7 @@
         <v>PASS</v>
       </c>
       <c r="H265">
-        <v>35</v>
+        <v>43</v>
       </c>
     </row>
     <row r="266">
@@ -7519,7 +7519,7 @@
         <v>PASS</v>
       </c>
       <c r="H266">
-        <v>57</v>
+        <v>52</v>
       </c>
     </row>
     <row r="267">
@@ -7545,7 +7545,7 @@
         <v>PASS</v>
       </c>
       <c r="H267">
-        <v>31</v>
+        <v>16</v>
       </c>
     </row>
     <row r="268">
@@ -7571,7 +7571,7 @@
         <v>PASS</v>
       </c>
       <c r="H268">
-        <v>27</v>
+        <v>46</v>
       </c>
     </row>
     <row r="269">
@@ -7597,7 +7597,7 @@
         <v>PASS</v>
       </c>
       <c r="H269">
-        <v>39</v>
+        <v>33</v>
       </c>
     </row>
     <row r="270">
@@ -7623,7 +7623,7 @@
         <v>PASS</v>
       </c>
       <c r="H270">
-        <v>27</v>
+        <v>58</v>
       </c>
     </row>
     <row r="271">
@@ -7649,7 +7649,7 @@
         <v>PASS</v>
       </c>
       <c r="H271">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="272" xml:space="preserve">
@@ -7676,7 +7676,7 @@
         <v>PASS</v>
       </c>
       <c r="H272">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="273">
@@ -7702,7 +7702,7 @@
         <v>PASS</v>
       </c>
       <c r="H273">
-        <v>34</v>
+        <v>38</v>
       </c>
     </row>
     <row r="274">
@@ -7728,7 +7728,7 @@
         <v>PASS</v>
       </c>
       <c r="H274">
-        <v>53</v>
+        <v>32</v>
       </c>
     </row>
     <row r="275">
@@ -7754,7 +7754,7 @@
         <v>PASS</v>
       </c>
       <c r="H275">
-        <v>24</v>
+        <v>50</v>
       </c>
     </row>
     <row r="276">
@@ -7780,7 +7780,7 @@
         <v>PASS</v>
       </c>
       <c r="H276">
-        <v>41</v>
+        <v>19</v>
       </c>
     </row>
     <row r="277">
@@ -7806,7 +7806,7 @@
         <v>PASS</v>
       </c>
       <c r="H277">
-        <v>21</v>
+        <v>54</v>
       </c>
     </row>
     <row r="278">
@@ -7832,7 +7832,7 @@
         <v>PASS</v>
       </c>
       <c r="H278">
-        <v>18</v>
+        <v>56</v>
       </c>
     </row>
     <row r="279" xml:space="preserve">
@@ -7859,7 +7859,7 @@
         <v>PASS</v>
       </c>
       <c r="H279">
-        <v>44</v>
+        <v>15</v>
       </c>
     </row>
     <row r="280">
@@ -7885,7 +7885,7 @@
         <v>PASS</v>
       </c>
       <c r="H280">
-        <v>54</v>
+        <v>58</v>
       </c>
     </row>
     <row r="281">
@@ -7911,7 +7911,7 @@
         <v>PASS</v>
       </c>
       <c r="H281">
-        <v>52</v>
+        <v>27</v>
       </c>
     </row>
     <row r="282">
@@ -7937,7 +7937,7 @@
         <v>PASS</v>
       </c>
       <c r="H282">
-        <v>39</v>
+        <v>52</v>
       </c>
     </row>
     <row r="283">
@@ -7963,7 +7963,7 @@
         <v>PASS</v>
       </c>
       <c r="H283">
-        <v>53</v>
+        <v>17</v>
       </c>
     </row>
     <row r="284">
@@ -7989,7 +7989,7 @@
         <v>PASS</v>
       </c>
       <c r="H284">
-        <v>38</v>
+        <v>31</v>
       </c>
     </row>
     <row r="285">
@@ -8015,7 +8015,7 @@
         <v>PASS</v>
       </c>
       <c r="H285">
-        <v>23</v>
+        <v>45</v>
       </c>
     </row>
     <row r="286">
@@ -8041,7 +8041,7 @@
         <v>PASS</v>
       </c>
       <c r="H286">
-        <v>21</v>
+        <v>39</v>
       </c>
     </row>
     <row r="287">
@@ -8067,7 +8067,7 @@
         <v>PASS</v>
       </c>
       <c r="H287">
-        <v>27</v>
+        <v>32</v>
       </c>
     </row>
     <row r="288">
@@ -8093,7 +8093,7 @@
         <v>PASS</v>
       </c>
       <c r="H288">
-        <v>47</v>
+        <v>58</v>
       </c>
     </row>
     <row r="289">
@@ -8119,7 +8119,7 @@
         <v>PASS</v>
       </c>
       <c r="H289">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="290">
@@ -8145,7 +8145,7 @@
         <v>PASS</v>
       </c>
       <c r="H290">
-        <v>39</v>
+        <v>53</v>
       </c>
     </row>
     <row r="291">
@@ -8171,7 +8171,7 @@
         <v>PASS</v>
       </c>
       <c r="H291">
-        <v>15</v>
+        <v>41</v>
       </c>
     </row>
     <row r="292">
@@ -8197,7 +8197,7 @@
         <v>PASS</v>
       </c>
       <c r="H292">
-        <v>22</v>
+        <v>57</v>
       </c>
     </row>
     <row r="293">
@@ -8223,7 +8223,7 @@
         <v>PASS</v>
       </c>
       <c r="H293">
-        <v>56</v>
+        <v>53</v>
       </c>
     </row>
     <row r="294">
@@ -8249,7 +8249,7 @@
         <v>PASS</v>
       </c>
       <c r="H294">
-        <v>44</v>
+        <v>23</v>
       </c>
     </row>
     <row r="295">
@@ -8275,7 +8275,7 @@
         <v>PASS</v>
       </c>
       <c r="H295">
-        <v>44</v>
+        <v>16</v>
       </c>
     </row>
     <row r="296">
@@ -8301,7 +8301,7 @@
         <v>PASS</v>
       </c>
       <c r="H296">
-        <v>38</v>
+        <v>47</v>
       </c>
     </row>
     <row r="297">
@@ -8327,7 +8327,7 @@
         <v>PASS</v>
       </c>
       <c r="H297">
-        <v>21</v>
+        <v>28</v>
       </c>
     </row>
     <row r="298">
@@ -8353,7 +8353,7 @@
         <v>PASS</v>
       </c>
       <c r="H298">
-        <v>53</v>
+        <v>23</v>
       </c>
     </row>
     <row r="299">
@@ -8379,7 +8379,7 @@
         <v>PASS</v>
       </c>
       <c r="H299">
-        <v>32</v>
+        <v>46</v>
       </c>
     </row>
     <row r="300">
@@ -8405,7 +8405,7 @@
         <v>PASS</v>
       </c>
       <c r="H300">
-        <v>59</v>
+        <v>54</v>
       </c>
     </row>
     <row r="301">
@@ -8431,7 +8431,7 @@
         <v>PASS</v>
       </c>
       <c r="H301">
-        <v>38</v>
+        <v>57</v>
       </c>
     </row>
   </sheetData>

</xml_diff>